<commit_message>
Achievement config table data Add ObjectPool
</commit_message>
<xml_diff>
--- a/Luban/DataTables/Datas/DesignPatternDataTable.xlsx
+++ b/Luban/DataTables/Datas/DesignPatternDataTable.xlsx
@@ -4,12 +4,12 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="27945" windowHeight="14175"/>
+    <workbookView windowWidth="27945" windowHeight="14175" activeTab="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Achievement" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
-    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
+    <sheet name="Achievement_Career" sheetId="1" r:id="rId1"/>
+    <sheet name="Achievement_Battle" sheetId="2" r:id="rId2"/>
+    <sheet name="Achievement_Area" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="56">
   <si>
     <t>##var</t>
   </si>
@@ -55,6 +55,9 @@
     <t>*achievement_rewards</t>
   </si>
   <si>
+    <t>strategy_type</t>
+  </si>
+  <si>
     <t>##type</t>
   </si>
   <si>
@@ -70,6 +73,9 @@
     <t>list,AchievementStageRewards</t>
   </si>
   <si>
+    <t>AchievementStrategyType</t>
+  </si>
+  <si>
     <t>##group</t>
   </si>
   <si>
@@ -103,6 +109,9 @@
     <t>成就奖励</t>
   </si>
   <si>
+    <t>成就策略类型</t>
+  </si>
+  <si>
     <t>生涯成就</t>
   </si>
   <si>
@@ -118,10 +127,76 @@
     <t>成就点,5|金币,100</t>
   </si>
   <si>
+    <t>QuantityReach</t>
+  </si>
+  <si>
     <t>成就点,5|金币,1000</t>
   </si>
   <si>
     <t>成就点,5|金币,10000</t>
+  </si>
+  <si>
+    <t>战斗成就</t>
+  </si>
+  <si>
+    <t>Boss达人-雷龙</t>
+  </si>
+  <si>
+    <t>雷龙猎杀者</t>
+  </si>
+  <si>
+    <t>击杀雷龙*次</t>
+  </si>
+  <si>
+    <t>BossKillCount</t>
+  </si>
+  <si>
+    <t>化险为夷·雷龙</t>
+  </si>
+  <si>
+    <t>血量低于10%，击杀雷龙*次</t>
+  </si>
+  <si>
+    <t>BossKillLowHp</t>
+  </si>
+  <si>
+    <t>id</t>
+  </si>
+  <si>
+    <t>category</t>
+  </si>
+  <si>
+    <t>parents</t>
+  </si>
+  <si>
+    <t>name</t>
+  </si>
+  <si>
+    <t>desc</t>
+  </si>
+  <si>
+    <t>*targets</t>
+  </si>
+  <si>
+    <t>*rewards</t>
+  </si>
+  <si>
+    <t>地区成就</t>
+  </si>
+  <si>
+    <t>格兰达·南部地区</t>
+  </si>
+  <si>
+    <t>欢迎来到格兰达</t>
+  </si>
+  <si>
+    <t>初次到达格兰达南部地区</t>
+  </si>
+  <si>
+    <t>探索专家</t>
+  </si>
+  <si>
+    <t>格兰达·南部地区探索度达到*%</t>
   </si>
 </sst>
 </file>
@@ -134,7 +209,7 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="21">
+  <fonts count="22">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -145,6 +220,12 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="等线"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="等线"/>
       <charset val="134"/>
     </font>
@@ -613,142 +694,145 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="2">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="4">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="5">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="4">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="6">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="7">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="12" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="15" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="16" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="19" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="20" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="21" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="22" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="23" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="24" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="25" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="27" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="28" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="29" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="30" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="31" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="32" borderId="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="4">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="5">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="4">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="6">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="7">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="8">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="10" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="11" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="12" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="13" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="14" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="15" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="16" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="17" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="18" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="19" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="20" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="21" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="22" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="23" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="24" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="25" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="26" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="27" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="28" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="29" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="30" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="31" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="32" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -1061,8 +1145,8 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:H7"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" outlineLevelRow="6" outlineLevelCol="7"/>
+  <dimension ref="A1:I7"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" outlineLevelRow="6"/>
   <cols>
     <col min="1" max="1" width="9" style="1"/>
     <col min="2" max="2" width="19.125" style="1" customWidth="1"/>
@@ -1072,10 +1156,11 @@
     <col min="6" max="6" width="43.25" style="1" customWidth="1"/>
     <col min="7" max="7" width="22.875" style="1" customWidth="1"/>
     <col min="8" max="8" width="27.25" style="1" customWidth="1"/>
-    <col min="9" max="16384" width="9" style="1"/>
+    <col min="9" max="9" width="22.875" style="1" customWidth="1"/>
+    <col min="10" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1" spans="1:8">
+    <row r="1" s="1" customFormat="1" spans="1:9">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1100,119 +1185,134 @@
       <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="2" s="1" customFormat="1" spans="1:8">
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" s="1" customFormat="1" spans="1:9">
       <c r="A2" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="3" s="1" customFormat="1" spans="1:8">
+        <v>13</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" s="1" customFormat="1" spans="1:9">
       <c r="A3" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="4" s="1" customFormat="1" spans="1:8">
+        <v>17</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4" s="1" customFormat="1" spans="1:9">
       <c r="A4" s="1" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="5" s="1" customFormat="1" spans="1:8">
+        <v>25</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="5" s="1" customFormat="1" spans="1:9">
       <c r="B5" s="1">
         <v>1</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="G5" s="1">
         <v>10000</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="6" s="1" customFormat="1" spans="1:8">
+        <v>31</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="6" s="1" customFormat="1" spans="1:9">
       <c r="G6" s="1">
         <v>100000</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9">
       <c r="G7" s="1">
         <v>1000000</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
     </row>
   </sheetData>
@@ -1225,9 +1325,219 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
-  <sheetData/>
+  <dimension ref="A1:I10"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
+  <cols>
+    <col min="1" max="1" width="9" style="1"/>
+    <col min="2" max="2" width="19.125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="20" style="1" customWidth="1"/>
+    <col min="4" max="4" width="14" style="1" customWidth="1"/>
+    <col min="5" max="5" width="28.125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="43.25" style="1" customWidth="1"/>
+    <col min="7" max="7" width="22.875" style="1" customWidth="1"/>
+    <col min="8" max="8" width="27.25" style="1" customWidth="1"/>
+    <col min="9" max="9" width="22.875" style="1" customWidth="1"/>
+    <col min="10" max="16384" width="9" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" s="1" customFormat="1" spans="1:9">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" s="1" customFormat="1" spans="1:9">
+      <c r="A2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" s="1" customFormat="1" spans="1:9">
+      <c r="A3" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4" s="1" customFormat="1" spans="1:9">
+      <c r="A4" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="5" s="1" customFormat="1" spans="1:9">
+      <c r="B5" s="1">
+        <v>100001</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="G5" s="1">
+        <v>10</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="6" s="1" customFormat="1" spans="1:9">
+      <c r="G6" s="1">
+        <v>20</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="7" s="1" customFormat="1" spans="1:9">
+      <c r="G7" s="1">
+        <v>30</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="8" s="1" customFormat="1" spans="1:9">
+      <c r="B8" s="1">
+        <v>100002</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="G8" s="1">
+        <v>1</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="9" s="1" customFormat="1" spans="1:9">
+      <c r="G9" s="1">
+        <v>5</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="10" s="1" customFormat="1" spans="1:9">
+      <c r="G10" s="1">
+        <v>10</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
   <headerFooter/>
@@ -1237,9 +1547,197 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
-  <sheetData/>
+  <dimension ref="A1:I8"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" outlineLevelRow="7"/>
+  <cols>
+    <col min="1" max="1" width="9" style="1"/>
+    <col min="2" max="2" width="19.125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="20" style="1" customWidth="1"/>
+    <col min="4" max="4" width="14" style="1" customWidth="1"/>
+    <col min="5" max="5" width="28.125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="43.25" style="1" customWidth="1"/>
+    <col min="7" max="7" width="22.875" style="1" customWidth="1"/>
+    <col min="8" max="8" width="27.25" style="1" customWidth="1"/>
+    <col min="9" max="9" width="22.875" style="1" customWidth="1"/>
+    <col min="10" max="16384" width="9" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" s="1" customFormat="1" spans="1:9">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" s="1" customFormat="1" spans="1:9">
+      <c r="A2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" s="1" customFormat="1" spans="1:9">
+      <c r="A3" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4" s="1" customFormat="1" spans="1:9">
+      <c r="A4" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="5" s="1" customFormat="1" spans="1:9">
+      <c r="B5" s="1">
+        <v>200001</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="G5" s="1">
+        <v>1</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="6" s="1" customFormat="1" spans="1:9">
+      <c r="B6" s="1">
+        <v>200002</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="G6" s="1">
+        <v>20</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="7" s="1" customFormat="1" spans="1:9">
+      <c r="G7" s="1">
+        <v>50</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="8" s="1" customFormat="1" spans="1:9">
+      <c r="G8" s="1">
+        <v>100</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
   <headerFooter/>

</xml_diff>